<commit_message>
latest fixes on the mirroring between starter and solution excel docs
</commit_message>
<xml_diff>
--- a/02_ai-risk-framework-implementation-nist-ai-rmf/exercises/solution/risk_assessment.xlsx
+++ b/02_ai-risk-framework-implementation-nist-ai-rmf/exercises/solution/risk_assessment.xlsx
@@ -594,7 +594,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>- EU AI Act: FraudShield classified as High-Risk for credit and fraud decisions</t>
+          <t>- EU AI Act: fraud-detection is exempt from Annex III 5(b) High-Risk classification; FraudShield is governed as High-Risk internally because its outputs can feed credit-limit and account-eligibility decisions</t>
         </is>
       </c>
     </row>
@@ -625,7 +625,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Identify all risks across NIST AI RMF categories (technical, ethical, legal, operational), populate the risk register with mitigation strategies, score risks, and generate an executive summary.</t>
+          <t>Identify all risks across the four risk categories (technical, ethical, legal, operational), map each to a NIST AI RMF function (Govern / Map / Measure / Manage), populate the risk register with mitigation strategies, score risks, and generate an executive summary.</t>
         </is>
       </c>
     </row>

</xml_diff>